<commit_message>
Update NandiSeedRecommender2 with new GEE data, suitability outputs, and refined notebooks
</commit_message>
<xml_diff>
--- a/02_NandiSeedRecommender2/Seed_Data/KenyaSeedWebScrape.xlsx
+++ b/02_NandiSeedRecommender2/Seed_Data/KenyaSeedWebScrape.xlsx
@@ -72,7 +72,7 @@
     <t>Moisture-Stress Tolerant</t>
   </si>
   <si>
-    <t>Lodging Resistance</t>
+    <t>Flood-Resistant</t>
   </si>
   <si>
     <t>Heat Tolerant</t>
@@ -549,7 +549,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="6" width="12.63"/>
+    <col customWidth="1" min="1" max="1" width="40.0"/>
     <col customWidth="1" min="8" max="9" width="35.0"/>
     <col customWidth="1" min="10" max="10" width="83.38"/>
   </cols>
@@ -582,7 +582,7 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -609,7 +609,7 @@
       <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
       <c r="T1" s="1" t="s">
@@ -816,8 +816,8 @@
       <c r="R4" s="1">
         <v>0.0</v>
       </c>
-      <c r="S4" s="1">
-        <v>0.0</v>
+      <c r="S4" s="2">
+        <v>1.0</v>
       </c>
       <c r="T4" s="1">
         <v>0.0</v>

</xml_diff>